<commit_message>
Always Positive Variance: The logic uses abs(val_a - val_b), so you will never see a negative dollar difference.
Precision Percentage: Calculated as (Difference / Ledger A) * 100, rounded to 2 decimals.

Professional Formatting: The export includes both Ledger A and Ledger B side-by-side for clear side-by-side verification.
</commit_message>
<xml_diff>
--- a/sample files for test/grouped_data.xlsx
+++ b/sample files for test/grouped_data.xlsx
@@ -52,13 +52,13 @@
     <t xml:space="preserve">Germany</t>
   </si>
   <si>
+    <t xml:space="preserve">Events</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Promotional</t>
+  </si>
+  <si>
     <t xml:space="preserve">Direct Contacts</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Events</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Promotional</t>
   </si>
 </sst>
 </file>
@@ -153,7 +153,7 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -355,8 +355,8 @@
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="3" min="3" style="1" width="15.27"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="4" min="4" style="1" width="24.47"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="5" style="1" width="23.56"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="26.59"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="25.69"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="1" width="26.58"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="7" min="7" style="1" width="25.7"/>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="8" min="8" style="1" width="14.77"/>
     <col collapsed="false" customWidth="false" hidden="false" outlineLevel="0" max="16384" min="9" style="1" width="11.53"/>
   </cols>
@@ -418,19 +418,19 @@
         <v>10</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>8183742</v>
+        <v>3099892</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>12795737</v>
+        <v>2214208</v>
       </c>
       <c r="F3" s="2" t="n">
-        <v>34256275</v>
+        <v>41099709</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>41440011</v>
+        <v>37261137</v>
       </c>
       <c r="H3" s="2" t="n">
-        <v>4.19</v>
+        <v>13.26</v>
       </c>
     </row>
     <row r="4" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -444,19 +444,19 @@
         <v>11</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>3099892</v>
+        <v>3281093</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>2214208</v>
+        <v>2506572</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>41099709</v>
+        <v>23166743</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>37261137</v>
+        <v>20881575</v>
       </c>
       <c r="H4" s="2" t="n">
-        <v>13.26</v>
+        <v>7.06</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="13.8" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -470,19 +470,19 @@
         <v>12</v>
       </c>
       <c r="D5" s="2" t="n">
-        <v>3281093</v>
+        <v>8183742</v>
       </c>
       <c r="E5" s="2" t="n">
-        <v>2506572</v>
+        <v>12795737</v>
       </c>
       <c r="F5" s="2" t="n">
-        <v>23166743</v>
+        <v>34256275</v>
       </c>
       <c r="G5" s="2" t="n">
-        <v>20881575</v>
+        <v>41440011</v>
       </c>
       <c r="H5" s="2" t="n">
-        <v>7.06</v>
+        <v>4.19</v>
       </c>
     </row>
   </sheetData>

</xml_diff>